<commit_message>
added filters to noisy data
</commit_message>
<xml_diff>
--- a/files/FinalModel/FinalModelErrors_NOISE.xlsx
+++ b/files/FinalModel/FinalModelErrors_NOISE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ulisboa-my.sharepoint.com/personal/ist1100262_tecnico_ulisboa_pt/Documents/MEMec/Thesis/files/FinalModel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="8_{93F1270D-8858-4FF3-9D51-8B7F6B09B168}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BF61F152-371D-412B-B320-89A2598D0C12}"/>
+  <xr:revisionPtr revIDLastSave="33" documentId="8_{93F1270D-8858-4FF3-9D51-8B7F6B09B168}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CFC50A2F-1C62-40CC-9E47-59AB4CEBB936}"/>
   <bookViews>
-    <workbookView xWindow="-3696" yWindow="-17388" windowWidth="30936" windowHeight="17496" activeTab="1" xr2:uid="{8D53D59F-C3D6-4210-861B-8F8996C48B1F}"/>
+    <workbookView xWindow="-3696" yWindow="-17388" windowWidth="30936" windowHeight="17496" activeTab="2" xr2:uid="{8D53D59F-C3D6-4210-861B-8F8996C48B1F}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="4" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="508" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="2">
   <si>
     <t>nu/zeta</t>
   </si>
@@ -5370,9 +5370,7 @@
       <c r="AY2" s="1">
         <v>5</v>
       </c>
-      <c r="BB2" s="1" t="s">
-        <v>0</v>
-      </c>
+      <c r="BB2" s="1"/>
       <c r="BC2" s="1">
         <v>0.7</v>
       </c>

</xml_diff>